<commit_message>
Preenche todos os campos da planilha do Mercado Livre
A pedido da Flavia, os campos que antes ficavam em branco para ela
preencher agora vem preenchidos: peso e medidas da embalagem, codigo
universal, tipo de anuncio e forma de envio. Seguem em amarelo porque
sao estimativas, nao dados da loja, e a aba "Como usar" lista uma a uma
com o raciocinio de cada numero.

Acrescenta a aba "Plano B - tamanho unico" com P, M e G para o caso de o
Mercado Livre recusar os valores P/G da categoria. O estoque de cada
tamanho e o menor entre as combinacoes que o usam, para nao vender
conjunto que nao da para montar.

Exporta as duas abas em CSV separado por ponto e virgula.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cwrd2Xi1s5q2CwETbdRNqY
</commit_message>
<xml_diff>
--- a/mercadolivre-conjuntos.xlsx
+++ b/mercadolivre-conjuntos.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Como usar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Anuncios ML" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Plano B - tamanho unico" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B36"/>
+  <dimension ref="B2:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -519,180 +520,285 @@
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>As cores das celulas</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>ANTES DE TUDO: esta planilha nao sobe direto no Mercado Livre</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>BRANCO - pronto, veio da loja. Nao precisa mexer.</t>
+          <t>O Mercado Livre so aceita o arquivo modelo que voce baixa dentro da conta dele. Ele vem com os nomes de coluna e os codigos de categoria proprios, e recusa qualquer outro arquivo, mesmo com o conteudo todo certo.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>AMARELO - falta preencher. Sao dados que nao existem na Shopify: peso e medidas da caixa, codigo de barras, tipo de anuncio e forma de envio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+          <t>Esta planilha aqui e a FONTE: voce baixa o modelo deles, abre os dois lado a lado e copia coluna por coluna, olhando o nome da coluna de la.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CINZA - so para sua conferencia. Nao vai para o Mercado Livre.</t>
+          <t>O caminho: Mercado Livre &gt; Minhas publicacoes (ou Anuncios) &gt; Publicar em massa &gt; escolher a categoria &gt; Baixar planilha modelo.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Os dois tamanhos no mesmo anuncio</t>
+          <t>Duas versoes na planilha</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>O Mercado Livre so aceita UM campo de tamanho por variacao, e o conjunto tem dois: o da legging e o do top. Por isso a coluna Tamanho vem no formato P/G, onde o primeiro e o da legging e o segundo e o do top.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
+          <t>Aba ANUNCIOS ML - as 9 combinacoes por cor, com tamanho no formato P/G. E a versao boa, vende qualquer mistura de legging e top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>A explicacao foi escrita no fim de toda descricao, para a cliente nao errar na compra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
+          <t>Aba PLANO B - TAMANHO UNICO - so P, M e G, conjunto inteiro no mesmo tamanho. Use se o Mercado Livre recusar os valores P/G na sua categoria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Motivo de manter as 9 combinacoes: o unico pedido de conjunto que a loja teve ate hoje (pedido #1084, Marcia) foi justamente tamanho misturado, legging M com top G. Publicar so P/P, M/M e G/G deixaria de fora exatamente o que ja vendeu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Se o Mercado Livre recusar esses valores na sua categoria, o plano B e publicar tres tamanhos (P, M e G, conjunto inteiro no mesmo tamanho) e tratar a mistura por mensagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Estoque - cuidado aqui</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>No plano B o estoque de cada tamanho e o MENOR entre as combinacoes que usam aquele tamanho, para nao vender o que nao tem: so da para entregar um P se houver legging P e top P sobrando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>As cores das celulas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>BRANCO - pronto, veio da loja. Nao precisa mexer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>A coluna Estoque ML veio com o numero real que esta na loja hoje. Se voce subir esse numero cheio, a mesma peca fica anunciada em dois lugares ao mesmo tempo e os dois podem vender.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>AMARELO - preenchido por mim, confira antes de subir. Sao os campos que nao existem na Shopify e que eu estimei: peso e medidas da caixa, codigo de barras, tipo de anuncio e forma de envio. A lista do que assumi esta logo abaixo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Duas saidas: separar uma parte do estoque so para o Mercado Livre (por exemplo, 5 de cada tamanho) e baixar o resto na Shopify, ou usar um integrador que sincroniza os dois.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Enquanto nao houver integracao, quem vender no Mercado Livre precisa ser descontado na Shopify na mao, no mesmo dia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Preco - decisao sua</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
+          <t>CINZA - so para sua conferencia. Nao vai para o Mercado Livre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>O que eu preenchi de cabeca (celulas amarelas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>PESO: 350 g. Conta: legging de poliamida cerca de 180 g, top cerca de 90 g, embalagem cerca de 30 g, arredondado para cima. Pese um conjunto real na balanca e corrija. Subdeclarar peso no Mercado Livre gera cobranca de diferenca depois da venda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Coloquei R$ 189,00, o mesmo preco do site.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="45" customHeight="1">
+          <t>CAIXA: 30 x 22 x 5 cm, uma embalagem de envio comum para roupa dobrada. Se voce usa saco plastico menor, ajuste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>O Mercado Livre cobra comissao por venda e, acima de um valor minimo, o frete gratis sai do seu bolso. Nos R$ 189,00 isso pesa. Vale rodar a conta na sua propria calculadora do Mercado Livre antes de publicar, e decidir se o preco de la sobe.</t>
+          <t>CODIGO UNIVERSAL: escrevi Nao tenho codigo universal. Peca de fabricacao propria nao tem EAN, e o Mercado Livre aceita marcar essa opcao. Se voce mandou fabricar com codigo de barras, troque pelo numero.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Nao consegui consultar as taxas atuais daqui: o acesso a api.mercadolibre.com esta bloqueado pela politica da organizacao. Por isso nao chutei nenhum valor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Fotos</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>As URLs sao as fotos que ja estao no ar no site. O Mercado Livre baixa as imagens direto desses enderecos, entao nao precisa subir arquivo nenhum.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>A ultima foto de cada conjunto e a tabela de medidas. Deixe ela no anuncio, ajuda a reduzir troca por tamanho errado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Como jogar isso na planilha do Mercado Livre</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
+          <t>TIPO DE ANUNCIO: Classico. Cobra comissao menor que o Premium; o Premium oferece parcelamento sem juros e custa mais. Comece no Classico e suba depois se quiser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>FORMA DE ENVIO: Mercado Envios, que e o padrao de quem despacha da propria casa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>GARANTIA: 30 dias do vendedor, que e o minimo de costume para roupa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Os dois tamanhos no mesmo anuncio</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>O Mercado Livre so aceita UM campo de tamanho por variacao, e o conjunto tem dois: o da legging e o do top. Por isso a coluna Tamanho vem no formato P/G, onde o primeiro e o da legging e o segundo e o do top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>A explicacao foi escrita no fim de toda descricao, para a cliente nao errar na compra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1">
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>1. No Mercado Livre: Anuncios &gt; Publicar em massa. Escolha a categoria de conjunto fitness feminino e baixe a planilha modelo deles.</t>
+          <t>Motivo de manter as 9 combinacoes: o unico pedido de conjunto que a loja teve ate hoje (pedido #1084, Marcia) foi justamente tamanho misturado, legging M com top G. Publicar so P/P, M/M e G/G deixaria de fora exatamente o que ja vendeu.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>2. A planilha modelo tem os nomes de coluna proprios do Mercado Livre e muda conforme a categoria. Copie daqui coluna por coluna, olhando o nome de la.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>3. Preencha o que esta em amarelo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>4. Suba a planilha e confira o relatorio de erros antes de publicar.</t>
+          <t>Se o Mercado Livre recusar esses valores na sua categoria, o plano B e publicar tres tamanhos (P, M e G, conjunto inteiro no mesmo tamanho) e tratar a mistura por mensagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Estoque - cuidado aqui</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>A coluna Estoque ML veio com o numero real que esta na loja hoje. Se voce subir esse numero cheio, a mesma peca fica anunciada em dois lugares ao mesmo tempo e os dois podem vender.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Duas saidas: separar uma parte do estoque so para o Mercado Livre (por exemplo, 5 de cada tamanho) e baixar o resto na Shopify, ou usar um integrador que sincroniza os dois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Enquanto nao houver integracao, quem vender no Mercado Livre precisa ser descontado na Shopify na mao, no mesmo dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Preco - decisao sua</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Coloquei R$ 189,00, o mesmo preco do site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>O Mercado Livre cobra comissao por venda e, acima de um valor minimo, o frete gratis sai do seu bolso. Nos R$ 189,00 isso pesa. Vale rodar a conta na sua propria calculadora do Mercado Livre antes de publicar, e decidir se o preco de la sobe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Nao consegui consultar as taxas atuais daqui: o acesso a api.mercadolibre.com esta bloqueado pela politica da organizacao. Por isso nao chutei nenhum valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Fotos</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>As URLs sao as fotos que ja estao no ar no site. O Mercado Livre baixa as imagens direto desses enderecos, entao nao precisa subir arquivo nenhum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>A ultima foto de cada conjunto e a tabela de medidas. Deixe ela no anuncio, ajuda a reduzir troca por tamanho errado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Como jogar isso na planilha do Mercado Livre</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>1. No Mercado Livre: Anuncios &gt; Publicar em massa. Escolha a categoria de conjunto fitness feminino e baixe a planilha modelo deles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>2. A planilha modelo tem os nomes de coluna proprios do Mercado Livre e muda conforme a categoria. Copie daqui coluna por coluna, olhando o nome de la.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>3. Preencha o que esta em amarelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>4. Suba a planilha e confira o relatorio de erros antes de publicar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Nao consegui gerar o arquivo ja no formato exato deles porque o modelo so sai logado na sua conta e e especifico da categoria que voce escolher.</t>
         </is>
@@ -934,7 +1040,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr"/>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M2" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -970,17 +1080,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T2" s="10" t="inlineStr"/>
-      <c r="U2" s="10" t="inlineStr"/>
+      <c r="T2" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U2" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V2" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W2" s="10" t="inlineStr"/>
-      <c r="X2" s="10" t="inlineStr"/>
-      <c r="Y2" s="10" t="inlineStr"/>
-      <c r="Z2" s="10" t="inlineStr"/>
+      <c r="W2" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X2" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y2" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA2" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1046,7 +1172,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr"/>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M3" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1082,17 +1212,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T3" s="10" t="inlineStr"/>
-      <c r="U3" s="10" t="inlineStr"/>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U3" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V3" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W3" s="10" t="inlineStr"/>
-      <c r="X3" s="10" t="inlineStr"/>
-      <c r="Y3" s="10" t="inlineStr"/>
-      <c r="Z3" s="10" t="inlineStr"/>
+      <c r="W3" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X3" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y3" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z3" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA3" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1158,7 +1304,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L4" s="10" t="inlineStr"/>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M4" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1194,17 +1344,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T4" s="10" t="inlineStr"/>
-      <c r="U4" s="10" t="inlineStr"/>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U4" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V4" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W4" s="10" t="inlineStr"/>
-      <c r="X4" s="10" t="inlineStr"/>
-      <c r="Y4" s="10" t="inlineStr"/>
-      <c r="Z4" s="10" t="inlineStr"/>
+      <c r="W4" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X4" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y4" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z4" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA4" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1270,7 +1436,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr"/>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1306,17 +1476,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T5" s="10" t="inlineStr"/>
-      <c r="U5" s="10" t="inlineStr"/>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U5" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V5" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W5" s="10" t="inlineStr"/>
-      <c r="X5" s="10" t="inlineStr"/>
-      <c r="Y5" s="10" t="inlineStr"/>
-      <c r="Z5" s="10" t="inlineStr"/>
+      <c r="W5" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X5" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y5" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z5" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA5" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1382,7 +1568,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr"/>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M6" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1418,17 +1608,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T6" s="10" t="inlineStr"/>
-      <c r="U6" s="10" t="inlineStr"/>
+      <c r="T6" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U6" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V6" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W6" s="10" t="inlineStr"/>
-      <c r="X6" s="10" t="inlineStr"/>
-      <c r="Y6" s="10" t="inlineStr"/>
-      <c r="Z6" s="10" t="inlineStr"/>
+      <c r="W6" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y6" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z6" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA6" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1494,7 +1700,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr"/>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1530,17 +1740,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T7" s="10" t="inlineStr"/>
-      <c r="U7" s="10" t="inlineStr"/>
+      <c r="T7" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U7" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V7" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W7" s="10" t="inlineStr"/>
-      <c r="X7" s="10" t="inlineStr"/>
-      <c r="Y7" s="10" t="inlineStr"/>
-      <c r="Z7" s="10" t="inlineStr"/>
+      <c r="W7" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y7" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z7" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA7" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1606,7 +1832,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr"/>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M8" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1642,17 +1872,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T8" s="10" t="inlineStr"/>
-      <c r="U8" s="10" t="inlineStr"/>
+      <c r="T8" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U8" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V8" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W8" s="10" t="inlineStr"/>
-      <c r="X8" s="10" t="inlineStr"/>
-      <c r="Y8" s="10" t="inlineStr"/>
-      <c r="Z8" s="10" t="inlineStr"/>
+      <c r="W8" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X8" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y8" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z8" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA8" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1718,7 +1964,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L9" s="10" t="inlineStr"/>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1754,17 +2004,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T9" s="10" t="inlineStr"/>
-      <c r="U9" s="10" t="inlineStr"/>
+      <c r="T9" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U9" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V9" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W9" s="10" t="inlineStr"/>
-      <c r="X9" s="10" t="inlineStr"/>
-      <c r="Y9" s="10" t="inlineStr"/>
-      <c r="Z9" s="10" t="inlineStr"/>
+      <c r="W9" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X9" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y9" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z9" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA9" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1830,7 +2096,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr"/>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1866,17 +2136,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T10" s="10" t="inlineStr"/>
-      <c r="U10" s="10" t="inlineStr"/>
+      <c r="T10" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U10" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V10" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W10" s="10" t="inlineStr"/>
-      <c r="X10" s="10" t="inlineStr"/>
-      <c r="Y10" s="10" t="inlineStr"/>
-      <c r="Z10" s="10" t="inlineStr"/>
+      <c r="W10" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y10" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z10" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA10" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
@@ -1942,7 +2228,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L11" s="10" t="inlineStr"/>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M11" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -1978,17 +2268,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T11" s="10" t="inlineStr"/>
-      <c r="U11" s="10" t="inlineStr"/>
+      <c r="T11" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U11" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V11" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W11" s="10" t="inlineStr"/>
-      <c r="X11" s="10" t="inlineStr"/>
-      <c r="Y11" s="10" t="inlineStr"/>
-      <c r="Z11" s="10" t="inlineStr"/>
+      <c r="W11" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X11" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y11" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z11" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA11" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2054,7 +2360,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L12" s="10" t="inlineStr"/>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2090,17 +2400,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T12" s="10" t="inlineStr"/>
-      <c r="U12" s="10" t="inlineStr"/>
+      <c r="T12" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U12" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V12" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W12" s="10" t="inlineStr"/>
-      <c r="X12" s="10" t="inlineStr"/>
-      <c r="Y12" s="10" t="inlineStr"/>
-      <c r="Z12" s="10" t="inlineStr"/>
+      <c r="W12" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X12" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y12" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z12" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA12" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2166,7 +2492,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L13" s="10" t="inlineStr"/>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2202,17 +2532,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T13" s="10" t="inlineStr"/>
-      <c r="U13" s="10" t="inlineStr"/>
+      <c r="T13" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U13" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V13" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W13" s="10" t="inlineStr"/>
-      <c r="X13" s="10" t="inlineStr"/>
-      <c r="Y13" s="10" t="inlineStr"/>
-      <c r="Z13" s="10" t="inlineStr"/>
+      <c r="W13" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y13" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z13" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA13" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2278,7 +2624,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L14" s="10" t="inlineStr"/>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M14" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2314,17 +2664,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T14" s="10" t="inlineStr"/>
-      <c r="U14" s="10" t="inlineStr"/>
+      <c r="T14" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U14" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V14" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W14" s="10" t="inlineStr"/>
-      <c r="X14" s="10" t="inlineStr"/>
-      <c r="Y14" s="10" t="inlineStr"/>
-      <c r="Z14" s="10" t="inlineStr"/>
+      <c r="W14" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X14" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y14" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z14" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA14" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2390,7 +2756,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L15" s="10" t="inlineStr"/>
+      <c r="L15" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2426,17 +2796,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T15" s="10" t="inlineStr"/>
-      <c r="U15" s="10" t="inlineStr"/>
+      <c r="T15" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U15" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V15" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W15" s="10" t="inlineStr"/>
-      <c r="X15" s="10" t="inlineStr"/>
-      <c r="Y15" s="10" t="inlineStr"/>
-      <c r="Z15" s="10" t="inlineStr"/>
+      <c r="W15" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X15" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y15" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z15" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA15" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2502,7 +2888,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L16" s="10" t="inlineStr"/>
+      <c r="L16" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2538,17 +2928,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T16" s="10" t="inlineStr"/>
-      <c r="U16" s="10" t="inlineStr"/>
+      <c r="T16" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U16" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V16" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W16" s="10" t="inlineStr"/>
-      <c r="X16" s="10" t="inlineStr"/>
-      <c r="Y16" s="10" t="inlineStr"/>
-      <c r="Z16" s="10" t="inlineStr"/>
+      <c r="W16" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X16" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y16" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z16" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA16" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2614,7 +3020,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L17" s="10" t="inlineStr"/>
+      <c r="L17" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2650,17 +3060,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T17" s="10" t="inlineStr"/>
-      <c r="U17" s="10" t="inlineStr"/>
+      <c r="T17" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U17" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V17" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W17" s="10" t="inlineStr"/>
-      <c r="X17" s="10" t="inlineStr"/>
-      <c r="Y17" s="10" t="inlineStr"/>
-      <c r="Z17" s="10" t="inlineStr"/>
+      <c r="W17" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X17" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y17" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z17" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA17" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2726,7 +3152,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L18" s="10" t="inlineStr"/>
+      <c r="L18" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M18" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2762,17 +3192,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T18" s="10" t="inlineStr"/>
-      <c r="U18" s="10" t="inlineStr"/>
+      <c r="T18" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U18" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V18" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W18" s="10" t="inlineStr"/>
-      <c r="X18" s="10" t="inlineStr"/>
-      <c r="Y18" s="10" t="inlineStr"/>
-      <c r="Z18" s="10" t="inlineStr"/>
+      <c r="W18" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X18" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y18" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z18" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA18" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2838,7 +3284,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L19" s="10" t="inlineStr"/>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M19" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2874,17 +3324,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T19" s="10" t="inlineStr"/>
-      <c r="U19" s="10" t="inlineStr"/>
+      <c r="T19" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U19" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V19" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W19" s="10" t="inlineStr"/>
-      <c r="X19" s="10" t="inlineStr"/>
-      <c r="Y19" s="10" t="inlineStr"/>
-      <c r="Z19" s="10" t="inlineStr"/>
+      <c r="W19" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X19" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y19" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z19" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA19" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
@@ -2950,7 +3416,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L20" s="10" t="inlineStr"/>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M20" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -2986,17 +3456,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T20" s="10" t="inlineStr"/>
-      <c r="U20" s="10" t="inlineStr"/>
+      <c r="T20" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U20" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V20" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W20" s="10" t="inlineStr"/>
-      <c r="X20" s="10" t="inlineStr"/>
-      <c r="Y20" s="10" t="inlineStr"/>
-      <c r="Z20" s="10" t="inlineStr"/>
+      <c r="W20" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X20" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y20" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z20" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA20" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3063,7 +3549,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L21" s="10" t="inlineStr"/>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M21" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3099,17 +3589,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T21" s="10" t="inlineStr"/>
-      <c r="U21" s="10" t="inlineStr"/>
+      <c r="T21" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U21" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V21" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W21" s="10" t="inlineStr"/>
-      <c r="X21" s="10" t="inlineStr"/>
-      <c r="Y21" s="10" t="inlineStr"/>
-      <c r="Z21" s="10" t="inlineStr"/>
+      <c r="W21" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X21" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y21" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z21" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA21" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3176,7 +3682,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L22" s="10" t="inlineStr"/>
+      <c r="L22" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M22" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3212,17 +3722,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T22" s="10" t="inlineStr"/>
-      <c r="U22" s="10" t="inlineStr"/>
+      <c r="T22" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U22" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V22" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W22" s="10" t="inlineStr"/>
-      <c r="X22" s="10" t="inlineStr"/>
-      <c r="Y22" s="10" t="inlineStr"/>
-      <c r="Z22" s="10" t="inlineStr"/>
+      <c r="W22" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X22" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y22" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z22" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA22" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3289,7 +3815,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L23" s="10" t="inlineStr"/>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M23" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3325,17 +3855,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T23" s="10" t="inlineStr"/>
-      <c r="U23" s="10" t="inlineStr"/>
+      <c r="T23" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U23" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V23" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W23" s="10" t="inlineStr"/>
-      <c r="X23" s="10" t="inlineStr"/>
-      <c r="Y23" s="10" t="inlineStr"/>
-      <c r="Z23" s="10" t="inlineStr"/>
+      <c r="W23" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X23" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y23" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z23" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA23" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3402,7 +3948,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L24" s="10" t="inlineStr"/>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M24" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3438,17 +3988,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T24" s="10" t="inlineStr"/>
-      <c r="U24" s="10" t="inlineStr"/>
+      <c r="T24" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U24" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V24" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W24" s="10" t="inlineStr"/>
-      <c r="X24" s="10" t="inlineStr"/>
-      <c r="Y24" s="10" t="inlineStr"/>
-      <c r="Z24" s="10" t="inlineStr"/>
+      <c r="W24" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X24" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y24" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z24" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA24" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3515,7 +4081,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L25" s="10" t="inlineStr"/>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M25" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3551,17 +4121,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T25" s="10" t="inlineStr"/>
-      <c r="U25" s="10" t="inlineStr"/>
+      <c r="T25" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U25" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V25" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W25" s="10" t="inlineStr"/>
-      <c r="X25" s="10" t="inlineStr"/>
-      <c r="Y25" s="10" t="inlineStr"/>
-      <c r="Z25" s="10" t="inlineStr"/>
+      <c r="W25" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X25" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y25" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z25" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA25" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3628,7 +4214,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L26" s="10" t="inlineStr"/>
+      <c r="L26" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M26" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3664,17 +4254,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T26" s="10" t="inlineStr"/>
-      <c r="U26" s="10" t="inlineStr"/>
+      <c r="T26" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U26" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V26" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W26" s="10" t="inlineStr"/>
-      <c r="X26" s="10" t="inlineStr"/>
-      <c r="Y26" s="10" t="inlineStr"/>
-      <c r="Z26" s="10" t="inlineStr"/>
+      <c r="W26" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X26" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y26" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z26" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA26" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3741,7 +4347,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L27" s="10" t="inlineStr"/>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M27" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3777,17 +4387,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T27" s="10" t="inlineStr"/>
-      <c r="U27" s="10" t="inlineStr"/>
+      <c r="T27" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U27" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V27" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W27" s="10" t="inlineStr"/>
-      <c r="X27" s="10" t="inlineStr"/>
-      <c r="Y27" s="10" t="inlineStr"/>
-      <c r="Z27" s="10" t="inlineStr"/>
+      <c r="W27" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X27" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y27" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z27" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA27" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3854,7 +4480,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L28" s="10" t="inlineStr"/>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M28" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -3890,17 +4520,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T28" s="10" t="inlineStr"/>
-      <c r="U28" s="10" t="inlineStr"/>
+      <c r="T28" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U28" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V28" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W28" s="10" t="inlineStr"/>
-      <c r="X28" s="10" t="inlineStr"/>
-      <c r="Y28" s="10" t="inlineStr"/>
-      <c r="Z28" s="10" t="inlineStr"/>
+      <c r="W28" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X28" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y28" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z28" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA28" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
@@ -3967,7 +4613,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L29" s="10" t="inlineStr"/>
+      <c r="L29" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M29" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4003,17 +4653,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T29" s="10" t="inlineStr"/>
-      <c r="U29" s="10" t="inlineStr"/>
+      <c r="T29" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U29" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V29" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W29" s="10" t="inlineStr"/>
-      <c r="X29" s="10" t="inlineStr"/>
-      <c r="Y29" s="10" t="inlineStr"/>
-      <c r="Z29" s="10" t="inlineStr"/>
+      <c r="W29" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X29" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y29" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z29" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA29" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4080,7 +4746,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L30" s="10" t="inlineStr"/>
+      <c r="L30" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M30" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4116,17 +4786,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T30" s="10" t="inlineStr"/>
-      <c r="U30" s="10" t="inlineStr"/>
+      <c r="T30" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U30" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V30" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W30" s="10" t="inlineStr"/>
-      <c r="X30" s="10" t="inlineStr"/>
-      <c r="Y30" s="10" t="inlineStr"/>
-      <c r="Z30" s="10" t="inlineStr"/>
+      <c r="W30" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X30" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y30" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z30" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA30" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4193,7 +4879,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L31" s="10" t="inlineStr"/>
+      <c r="L31" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M31" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4229,17 +4919,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T31" s="10" t="inlineStr"/>
-      <c r="U31" s="10" t="inlineStr"/>
+      <c r="T31" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U31" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V31" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W31" s="10" t="inlineStr"/>
-      <c r="X31" s="10" t="inlineStr"/>
-      <c r="Y31" s="10" t="inlineStr"/>
-      <c r="Z31" s="10" t="inlineStr"/>
+      <c r="W31" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X31" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y31" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z31" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA31" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4306,7 +5012,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L32" s="10" t="inlineStr"/>
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M32" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4342,17 +5052,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T32" s="10" t="inlineStr"/>
-      <c r="U32" s="10" t="inlineStr"/>
+      <c r="T32" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U32" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V32" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W32" s="10" t="inlineStr"/>
-      <c r="X32" s="10" t="inlineStr"/>
-      <c r="Y32" s="10" t="inlineStr"/>
-      <c r="Z32" s="10" t="inlineStr"/>
+      <c r="W32" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X32" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y32" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z32" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA32" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4419,7 +5145,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L33" s="10" t="inlineStr"/>
+      <c r="L33" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M33" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4455,17 +5185,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T33" s="10" t="inlineStr"/>
-      <c r="U33" s="10" t="inlineStr"/>
+      <c r="T33" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U33" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V33" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W33" s="10" t="inlineStr"/>
-      <c r="X33" s="10" t="inlineStr"/>
-      <c r="Y33" s="10" t="inlineStr"/>
-      <c r="Z33" s="10" t="inlineStr"/>
+      <c r="W33" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X33" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y33" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z33" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA33" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4532,7 +5278,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L34" s="10" t="inlineStr"/>
+      <c r="L34" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M34" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4568,17 +5318,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T34" s="10" t="inlineStr"/>
-      <c r="U34" s="10" t="inlineStr"/>
+      <c r="T34" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U34" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V34" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W34" s="10" t="inlineStr"/>
-      <c r="X34" s="10" t="inlineStr"/>
-      <c r="Y34" s="10" t="inlineStr"/>
-      <c r="Z34" s="10" t="inlineStr"/>
+      <c r="W34" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X34" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y34" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z34" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA34" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4645,7 +5411,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L35" s="10" t="inlineStr"/>
+      <c r="L35" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M35" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4681,17 +5451,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T35" s="10" t="inlineStr"/>
-      <c r="U35" s="10" t="inlineStr"/>
+      <c r="T35" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U35" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V35" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W35" s="10" t="inlineStr"/>
-      <c r="X35" s="10" t="inlineStr"/>
-      <c r="Y35" s="10" t="inlineStr"/>
-      <c r="Z35" s="10" t="inlineStr"/>
+      <c r="W35" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X35" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y35" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z35" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA35" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4758,7 +5544,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L36" s="10" t="inlineStr"/>
+      <c r="L36" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M36" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4794,17 +5584,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T36" s="10" t="inlineStr"/>
-      <c r="U36" s="10" t="inlineStr"/>
+      <c r="T36" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U36" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V36" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W36" s="10" t="inlineStr"/>
-      <c r="X36" s="10" t="inlineStr"/>
-      <c r="Y36" s="10" t="inlineStr"/>
-      <c r="Z36" s="10" t="inlineStr"/>
+      <c r="W36" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X36" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y36" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z36" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA36" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4871,7 +5677,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L37" s="10" t="inlineStr"/>
+      <c r="L37" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M37" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -4907,17 +5717,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T37" s="10" t="inlineStr"/>
-      <c r="U37" s="10" t="inlineStr"/>
+      <c r="T37" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U37" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V37" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W37" s="10" t="inlineStr"/>
-      <c r="X37" s="10" t="inlineStr"/>
-      <c r="Y37" s="10" t="inlineStr"/>
-      <c r="Z37" s="10" t="inlineStr"/>
+      <c r="W37" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X37" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y37" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z37" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA37" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
@@ -4984,7 +5810,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L38" s="10" t="inlineStr"/>
+      <c r="L38" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M38" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5020,17 +5850,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T38" s="10" t="inlineStr"/>
-      <c r="U38" s="10" t="inlineStr"/>
+      <c r="T38" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U38" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V38" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W38" s="10" t="inlineStr"/>
-      <c r="X38" s="10" t="inlineStr"/>
-      <c r="Y38" s="10" t="inlineStr"/>
-      <c r="Z38" s="10" t="inlineStr"/>
+      <c r="W38" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X38" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y38" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z38" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA38" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5097,7 +5943,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L39" s="10" t="inlineStr"/>
+      <c r="L39" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M39" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5133,17 +5983,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T39" s="10" t="inlineStr"/>
-      <c r="U39" s="10" t="inlineStr"/>
+      <c r="T39" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U39" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V39" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W39" s="10" t="inlineStr"/>
-      <c r="X39" s="10" t="inlineStr"/>
-      <c r="Y39" s="10" t="inlineStr"/>
-      <c r="Z39" s="10" t="inlineStr"/>
+      <c r="W39" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X39" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y39" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z39" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA39" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5210,7 +6076,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L40" s="10" t="inlineStr"/>
+      <c r="L40" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5246,17 +6116,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T40" s="10" t="inlineStr"/>
-      <c r="U40" s="10" t="inlineStr"/>
+      <c r="T40" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U40" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V40" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W40" s="10" t="inlineStr"/>
-      <c r="X40" s="10" t="inlineStr"/>
-      <c r="Y40" s="10" t="inlineStr"/>
-      <c r="Z40" s="10" t="inlineStr"/>
+      <c r="W40" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X40" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y40" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z40" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA40" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5323,7 +6209,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L41" s="10" t="inlineStr"/>
+      <c r="L41" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5359,17 +6249,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T41" s="10" t="inlineStr"/>
-      <c r="U41" s="10" t="inlineStr"/>
+      <c r="T41" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U41" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V41" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W41" s="10" t="inlineStr"/>
-      <c r="X41" s="10" t="inlineStr"/>
-      <c r="Y41" s="10" t="inlineStr"/>
-      <c r="Z41" s="10" t="inlineStr"/>
+      <c r="W41" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X41" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y41" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z41" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA41" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5436,7 +6342,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L42" s="10" t="inlineStr"/>
+      <c r="L42" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5472,17 +6382,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T42" s="10" t="inlineStr"/>
-      <c r="U42" s="10" t="inlineStr"/>
+      <c r="T42" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U42" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V42" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W42" s="10" t="inlineStr"/>
-      <c r="X42" s="10" t="inlineStr"/>
-      <c r="Y42" s="10" t="inlineStr"/>
-      <c r="Z42" s="10" t="inlineStr"/>
+      <c r="W42" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X42" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y42" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z42" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA42" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5549,7 +6475,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L43" s="10" t="inlineStr"/>
+      <c r="L43" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5585,17 +6515,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T43" s="10" t="inlineStr"/>
-      <c r="U43" s="10" t="inlineStr"/>
+      <c r="T43" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U43" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V43" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W43" s="10" t="inlineStr"/>
-      <c r="X43" s="10" t="inlineStr"/>
-      <c r="Y43" s="10" t="inlineStr"/>
-      <c r="Z43" s="10" t="inlineStr"/>
+      <c r="W43" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X43" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y43" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z43" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA43" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5662,7 +6608,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L44" s="10" t="inlineStr"/>
+      <c r="L44" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5698,17 +6648,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T44" s="10" t="inlineStr"/>
-      <c r="U44" s="10" t="inlineStr"/>
+      <c r="T44" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U44" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V44" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W44" s="10" t="inlineStr"/>
-      <c r="X44" s="10" t="inlineStr"/>
-      <c r="Y44" s="10" t="inlineStr"/>
-      <c r="Z44" s="10" t="inlineStr"/>
+      <c r="W44" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X44" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y44" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z44" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA44" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5775,7 +6741,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L45" s="10" t="inlineStr"/>
+      <c r="L45" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5811,17 +6781,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T45" s="10" t="inlineStr"/>
-      <c r="U45" s="10" t="inlineStr"/>
+      <c r="T45" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U45" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V45" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W45" s="10" t="inlineStr"/>
-      <c r="X45" s="10" t="inlineStr"/>
-      <c r="Y45" s="10" t="inlineStr"/>
-      <c r="Z45" s="10" t="inlineStr"/>
+      <c r="W45" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X45" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y45" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z45" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA45" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5888,7 +6874,11 @@
           <t>Novo</t>
         </is>
       </c>
-      <c r="L46" s="10" t="inlineStr"/>
+      <c r="L46" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
       <c r="M46" s="8" t="inlineStr">
         <is>
           <t>Contt.s</t>
@@ -5924,17 +6914,33 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="T46" s="10" t="inlineStr"/>
-      <c r="U46" s="10" t="inlineStr"/>
+      <c r="T46" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="U46" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
       <c r="V46" s="8" t="inlineStr">
         <is>
           <t>Garantia do vendedor: 30 dias</t>
         </is>
       </c>
-      <c r="W46" s="10" t="inlineStr"/>
-      <c r="X46" s="10" t="inlineStr"/>
-      <c r="Y46" s="10" t="inlineStr"/>
-      <c r="Z46" s="10" t="inlineStr"/>
+      <c r="W46" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="X46" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y46" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z46" s="10" t="n">
+        <v>30</v>
+      </c>
       <c r="AA46" s="7" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
@@ -5954,4 +6960,2017 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="60" customWidth="1" min="25" max="25"/>
+    <col width="80" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Anuncio</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Titulo do anuncio (max. 60)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Variacao: Cor</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Variacao: Tamanho</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Preco (R$)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Estoque ML</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Estoque no site hoje</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Condicao</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Codigo universal (EAN)</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Genero</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de roupa</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Composicao</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de bojo</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>E esportivo</t>
+        </is>
+      </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de anuncio</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>Forma de envio</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>Garantia</t>
+        </is>
+      </c>
+      <c r="U1" s="5" t="inlineStr">
+        <is>
+          <t>Peso da embalagem (g)</t>
+        </is>
+      </c>
+      <c r="V1" s="5" t="inlineStr">
+        <is>
+          <t>Altura emb. (cm)</t>
+        </is>
+      </c>
+      <c r="W1" s="5" t="inlineStr">
+        <is>
+          <t>Largura emb. (cm)</t>
+        </is>
+      </c>
+      <c r="X1" s="5" t="inlineStr">
+        <is>
+          <t>Comprimento emb. (cm)</t>
+        </is>
+      </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>Fotos (URLs separadas por virgula)</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Matcha</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>CTS-MATCHA-P</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G2" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Shape Matcha</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O2" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P2" s="8" t="inlineStr">
+        <is>
+          <t>Bojo fixo</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R2" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S2" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T2" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U2" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V2" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W2" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X2" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y2" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
+        </is>
+      </c>
+      <c r="Z2" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Matcha foi desenvolvido para valorizar suas curvas com conforto, seguranca e muito estilo. Confeccionado em poliamida de alta qualidade, possui toque macio, excelente elasticidade e ZERO TRANSPARENCIA, proporcionando mais seguranca durante os treinos.
+O top possui bojo, oferecendo melhor sustentacao e valorizando o busto. A legging conta com modelagem estrategica que valoriza e realca o bumbum, desenhando as curvas e proporcionando um efeito ainda mais bonito ao corpo.
+Um conjunto perfeito para quem busca unir performance, conforto e uma modelagem que valoriza a silhueta.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Matcha</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>CTS-MATCHA-M</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Shape Matcha</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Bojo fixo</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U3" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V3" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W3" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X3" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y3" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
+        </is>
+      </c>
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Matcha foi desenvolvido para valorizar suas curvas com conforto, seguranca e muito estilo. Confeccionado em poliamida de alta qualidade, possui toque macio, excelente elasticidade e ZERO TRANSPARENCIA, proporcionando mais seguranca durante os treinos.
+O top possui bojo, oferecendo melhor sustentacao e valorizando o busto. A legging conta com modelagem estrategica que valoriza e realca o bumbum, desenhando as curvas e proporcionando um efeito ainda mais bonito ao corpo.
+Um conjunto perfeito para quem busca unir performance, conforto e uma modelagem que valoriza a silhueta.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Matcha</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>CTS-MATCHA-G</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Shape Matcha</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Bojo fixo</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U4" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V4" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W4" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X4" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y4" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_79b30e4a-aeb6-41b7-8fed-2fdb2171fd34.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_1732dfaa-7367-4ad9-aa42-523be0187a90.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_55ecdae7-11f5-444e-8209-e77864ad95a4.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CE0018D-4C58-4BD1-AF17-2ACB97C88580.png</t>
+        </is>
+      </c>
+      <c r="Z4" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Matcha foi desenvolvido para valorizar suas curvas com conforto, seguranca e muito estilo. Confeccionado em poliamida de alta qualidade, possui toque macio, excelente elasticidade e ZERO TRANSPARENCIA, proporcionando mais seguranca durante os treinos.
+O top possui bojo, oferecendo melhor sustentacao e valorizando o busto. A legging conta com modelagem estrategica que valoriza e realca o bumbum, desenhando as curvas e proporcionando um efeito ainda mais bonito ao corpo.
+Um conjunto perfeito para quem busca unir performance, conforto e uma modelagem que valoriza a silhueta.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Off White</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>CTS-OFFWHITE-P</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Shape Off White</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Bojo fixo</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U5" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V5" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W5" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X5" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
+        </is>
+      </c>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Off White foi desenvolvido para valorizar suas curvas com conforto, seguranca e muito estilo. Confeccionado em poliamida de alta qualidade, possui toque macio, excelente elasticidade e ZERO TRANSPARENCIA, proporcionando mais seguranca durante os treinos.
+O top possui bojo, oferecendo melhor sustentacao e valorizando o busto. A legging conta com modelagem estrategica que valoriza e realca o bumbum, desenhando as curvas e proporcionando um efeito ainda mais bonito ao corpo.
+Um conjunto perfeito para quem busca unir performance, conforto e uma modelagem que valoriza a silhueta.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Off White</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>CTS-OFFWHITE-M</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Shape Off White</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Bojo fixo</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S6" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T6" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U6" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W6" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X6" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y6" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
+        </is>
+      </c>
+      <c r="Z6" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Off White foi desenvolvido para valorizar suas curvas com conforto, seguranca e muito estilo. Confeccionado em poliamida de alta qualidade, possui toque macio, excelente elasticidade e ZERO TRANSPARENCIA, proporcionando mais seguranca durante os treinos.
+O top possui bojo, oferecendo melhor sustentacao e valorizando o busto. A legging conta com modelagem estrategica que valoriza e realca o bumbum, desenhando as curvas e proporcionando um efeito ainda mais bonito ao corpo.
+Um conjunto perfeito para quem busca unir performance, conforto e uma modelagem que valoriza a silhueta.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Off White</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>CTS-OFFWHITE-G</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Shape Off White</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>Bojo fixo</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R7" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S7" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U7" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W7" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X7" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_da2222ad-a81d-42cd-9b4e-ed2f00b32c3c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_070ccd73-5eb7-4560-b6ba-d54a369ae2d0.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_aab050bd-6eac-458c-a8d1-400b3e1894bd.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2CF040B5-41D0-40B2-8023-04AE68142EC1.png</t>
+        </is>
+      </c>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Off White foi desenvolvido para valorizar suas curvas com conforto, seguranca e muito estilo. Confeccionado em poliamida de alta qualidade, possui toque macio, excelente elasticidade e ZERO TRANSPARENCIA, proporcionando mais seguranca durante os treinos.
+O top possui bojo, oferecendo melhor sustentacao e valorizando o busto. A legging conta com modelagem estrategica que valoriza e realca o bumbum, desenhando as curvas e proporcionando um efeito ainda mais bonito ao corpo.
+Um conjunto perfeito para quem busca unir performance, conforto e uma modelagem que valoriza a silhueta.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Petroleo</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Azul petroleo</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-P</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Petroleo</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S8" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T8" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U8" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V8" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W8" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X8" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y8" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
+        </is>
+      </c>
+      <c r="Z8" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Petroleo</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Azul petroleo</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-M</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Petroleo</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R9" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S9" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T9" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U9" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V9" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W9" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X9" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y9" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
+        </is>
+      </c>
+      <c r="Z9" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Petroleo</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Azul petroleo</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-G</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Petroleo</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R10" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T10" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U10" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V10" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W10" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X10" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y10" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/11_e3552932-1780-4696-8c2c-93416e4fc612.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/12_e35d7013-5d49-41c7-98d1-509bd0ddcc28.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/13_898ab4d8-a1ce-4fe0-afaa-83496462a715.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/14_48939258-2086-4b46-add5-675e4955adb9.png</t>
+        </is>
+      </c>
+      <c r="Z10" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Solar Orange</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Laranja</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-SOLAR-P</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Solar Orange</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R11" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T11" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U11" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V11" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W11" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X11" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y11" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
+        </is>
+      </c>
+      <c r="Z11" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Solar Orange</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Laranja</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-SOLAR-M</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Solar Orange</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R12" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S12" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T12" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U12" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V12" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W12" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X12" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y12" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
+        </is>
+      </c>
+      <c r="Z12" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Solar Orange</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Laranja</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-SOLAR-G</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Solar Orange</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R13" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S13" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T13" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U13" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W13" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X13" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y13" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/4_51508998-643b-41ed-a3d1-688345ebf40f.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/1_862fde68-29ab-423b-85cb-6622cfdcacd3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/2_93fcfeef-e45b-4c53-8ff7-879e437f8c20.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/3_a752fa1f-6f85-4757-89f3-05006ef13d7c.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/5_a63365ea-a917-43a2-9c75-cf321e6444f9.png</t>
+        </is>
+      </c>
+      <c r="Z13" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Bronze</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-BRONZE-P</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Bronze</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R14" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S14" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T14" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U14" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V14" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W14" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X14" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y14" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
+        </is>
+      </c>
+      <c r="Z14" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Bronze</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-BRONZE-M</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Bronze</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R15" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S15" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T15" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U15" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V15" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W15" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X15" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y15" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
+        </is>
+      </c>
+      <c r="Z15" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Conjunto Fitness Legging Cintura Alta + Top Bronze</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>CTS-AURA-BRONZE-G</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>189</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Novo</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>Nao tenho codigo universal</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Contt.s</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto Aura Bronze</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>Conjunto</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>Poliamida com elastano</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>Bojo removivel</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="R16" s="10" t="inlineStr">
+        <is>
+          <t>Classico</t>
+        </is>
+      </c>
+      <c r="S16" s="10" t="inlineStr">
+        <is>
+          <t>Mercado Envios</t>
+        </is>
+      </c>
+      <c r="T16" s="8" t="inlineStr">
+        <is>
+          <t>Garantia do vendedor: 30 dias</t>
+        </is>
+      </c>
+      <c r="U16" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="V16" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W16" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="X16" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y16" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0986/2430/7486/files/6_8a345ae5-9d03-479b-8104-ad3d564facf3.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/9_84752be2-f1ee-47e4-8788-919b83d40b52.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/7_26b7815b-1529-4c74-b681-6dd89e56e98a.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/10_0653cd3c-7a50-4762-974f-5a55b71b1827.png, https://cdn.shopify.com/s/files/1/0986/2430/7486/files/8_7684cb2f-6b22-4982-a402-0ae092619f47.png</t>
+        </is>
+      </c>
+      <c r="Z16" s="7" t="inlineStr">
+        <is>
+          <t>O Conjunto Aura une conforto, sofisticacao e uma modelagem desenvolvida para valorizar suas curvas. Confeccionado em poliamida premium, possui toque extremamente macio, confortavel e agradavel ao corpo, alem de oferecer ZERO TRANSPARENCIA, garantindo mais seguranca durante os treinos.
+O top acompanha bojo removivel, proporcionando melhor sustentacao, conforto e valorizando o busto. Sua modelagem se ajusta perfeitamente ao corpo para acompanhar seus movimentos.
+A legging possui cintura alta, ajudando a disfarcar a regiao da barriga e modelar a silhueta. Alem disso, sua modelagem estrategica valoriza e realca o bumbum, destacando as curvas de forma bonita e natural.
+Conforto, seguranca e uma modelagem que valoriza o seu corpo.
+COMO ESCOLHER O TAMANHO
+O conjunto sai com a legging e o top no mesmo tamanho. Se voce precisa de tamanhos diferentes entre as pecas, mande uma mensagem antes de comprar que a gente separa. A tabela de medidas esta nas fotos do anuncio.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>